<commit_message>
MO-517: add welsh translations
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/csoc/xlsx/01-csoc-account-home.xlsx
+++ b/translations/welsh-translations/csoc/xlsx/01-csoc-account-home.xlsx
@@ -76,7 +76,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="5" width="24" customWidth="1" hidden="1"/>
@@ -150,17 +150,17 @@
     <row r="6" ht="48" customHeight="1">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Csoc/_LandingBullet.en.resx::bullet_compliance_scheme</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_ManageRecyclingObligationsTile.en.resx::heading_direct_producer</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Csoc/_LandingBullet.en.resx</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_ManageRecyclingObligationsTile.en.resx</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">bullet_compliance_scheme</t>
+          <t xml:space="preserve">heading_direct_producer</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -175,12 +175,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve">submit your statement of compliance</t>
+          <t xml:space="preserve">Manage your {0} recycling obligations</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Rheoli'ch rhwymedigaethau ailgylchu ar gyfer {0}</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -192,17 +192,17 @@
     <row r="7" ht="48" customHeight="1">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Csoc/_LandingBullet.en.resx::bullet_direct_producer</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_ManageRecyclingObligationsTile.en.resx::heading_compliance_scheme</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Csoc/_LandingBullet.en.resx</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_ManageRecyclingObligationsTile.en.resx</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">bullet_direct_producer</t>
+          <t xml:space="preserve">heading_compliance_scheme</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -217,12 +217,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve">submit your certificate of compliance</t>
+          <t xml:space="preserve">Manage your {0} recycling obligations</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Rheoli'ch rhwymedigaethau ailgylchu ar gyfer {0}</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -234,17 +234,17 @@
     <row r="8" ht="48" customHeight="1">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Csoc/_LandingParagraph.en.resx::paragraph_compliance_scheme</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_ManageRecyclingObligationsTile.en.resx::paragraph_1_direct_producer</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Csoc/_LandingParagraph.en.resx</t>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_ManageRecyclingObligationsTile.en.resx</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">paragraph_compliance_scheme</t>
+          <t xml:space="preserve">paragraph_1_direct_producer</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -259,7 +259,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve">An approved or delegated person must submit your statement of compliance before or on &lt;strong&gt;{0:d MMMM yyyy}&lt;/strong&gt;.</t>
+          <t xml:space="preserve">Review your recycling obligations and accept PRNs or PERNs to meet them. You can also:</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -276,47 +276,383 @@
     <row r="9" ht="48" customHeight="1">
       <c r="A9" t="inlineStr">
         <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_ManageRecyclingObligationsTile.en.resx::paragraph_1_compliance_scheme</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_ManageRecyclingObligationsTile.en.resx</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">paragraph_1_compliance_scheme</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">csoc-account-home</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/report-data/home-compliance-scheme</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Review your recycling obligations and accept PRNs or PERNs to meet them. You can also:</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_ManageRecyclingObligationsTile.en.resx::unordered_list_point_1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_ManageRecyclingObligationsTile.en.resx</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unordered_list_point_1</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">csoc-account-home</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/report-data/home-compliance-scheme</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">see how your recycling obligations were calculated</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_ManageRecyclingObligationsTile.en.resx::unordered_list_point_2</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Prns/_ManageRecyclingObligationsTile.en.resx</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unordered_list_point_2</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">csoc-account-home</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/report-data/home-compliance-scheme</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">check your recycling obligations progress</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Csoc/_LandingBullet.en.resx::bullet_compliance_scheme</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Csoc/_LandingBullet.en.resx</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bullet_compliance_scheme</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">csoc-account-home</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/report-data/home-compliance-scheme</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">submit your statement of compliance</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cyflwyno eich datganiad cydymffurfio</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Csoc/_LandingBullet.en.resx::bullet_direct_producer</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Csoc/_LandingBullet.en.resx</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bullet_direct_producer</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">csoc-account-home</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/report-data/home-compliance-scheme</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">submit your certificate of compliance</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cyflwyno eich tystysgrif cydymffurfio</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Csoc/_LandingBullet.en.resx::bullet_view_compliance_scheme</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Csoc/_LandingBullet.en.resx</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bullet_view_compliance_scheme</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">csoc-account-home</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/report-data/home-compliance-scheme</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">view your statement of compliance</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gweld eich datganiad cydymffurfio</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Csoc/_LandingBullet.en.resx::bullet_view_direct_producer</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Csoc/_LandingBullet.en.resx</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bullet_view_direct_producer</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">csoc-account-home</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/report-data/home-compliance-scheme</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">view your certificate of compliance</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gweld eich tystysgrif cydymffurfio</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="48" customHeight="1">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Csoc/_LandingParagraph.en.resx::paragraph_compliance_scheme</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Csoc/_LandingParagraph.en.resx</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">paragraph_compliance_scheme</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">csoc-account-home</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/report-data/home-compliance-scheme</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">An approved or delegated person must submit your statement of compliance before or on {0:d MMMM yyyy}.</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rhaid i berson cymeradwy neu ddirprwyedig gyflwyno eich datganiad cydymffurfio ar {0:d MMMM yyyy} neu cyn hynny.</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1">
+      <c r="A17" t="inlineStr">
+        <is>
           <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Csoc/_LandingParagraph.en.resx::paragraph_direct_producer</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t xml:space="preserve">src/FrontendSchemeRegistration.UI/Resources/Views/Shared/Partials/Csoc/_LandingParagraph.en.resx</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t xml:space="preserve">paragraph_direct_producer</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">csoc-account-home</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">/report-data/home-compliance-scheme</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">An approved or delegated person must submit your certificate of compliance before or on &lt;strong&gt;{0:d MMMM yyyy}&lt;/strong&gt;.</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
+      <c r="D17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">csoc-account-home</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">/report-data/home-compliance-scheme</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">An approved or delegated person must submit your certificate of compliance before or on {0:d MMMM yyyy}.</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rhaid i berson cymeradwy neu ddirprwyedig gyflwyno eich tystysgrif cydymffurfio ar {0:d MMMM yyyy} neu cyn hynny.</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:H9"/>
+  <autoFilter ref="A5:H17"/>
   <mergeCells count="3">
     <mergeCell ref="F1:H1"/>
     <mergeCell ref="F2:H2"/>

</xml_diff>